<commit_message>
:sparkles: : Feat(bluemarble) :
1. 타일 정보 오타 수정

related: #458
</commit_message>
<xml_diff>
--- a/meeple_back/src/main/resources/game-element/bluemarble-tile.xlsx
+++ b/meeple_back/src/main/resources/game-element/bluemarble-tile.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10119"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SSAFY\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/biggie/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6B2840-3CE6-0947-B2C5-446197E50A8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15300" windowHeight="6860"/>
+    <workbookView xWindow="17180" yWindow="6280" windowWidth="25260" windowHeight="18700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="63">
   <si>
     <t>id</t>
   </si>
@@ -222,54 +223,53 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>백조자리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>헬리혜성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>헬리혜성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>수성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>yellow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>금성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>yellow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>뉴런의골짜기</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>백조자리</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>헬리혜성</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>헬리혜성</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>수성</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>yellow</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>금성</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>yellow</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -476,7 +476,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -753,11 +753,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E41"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -774,7 +774,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5">
         <v>0</v>
       </c>
@@ -787,7 +787,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -804,7 +804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -817,7 +817,7 @@
       </c>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -834,7 +834,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -851,7 +851,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -868,7 +868,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -885,7 +885,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -898,7 +898,7 @@
       </c>
       <c r="E9" s="8"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -915,7 +915,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -932,7 +932,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -940,10 +940,12 @@
         <v>20</v>
       </c>
       <c r="C12" s="6"/>
-      <c r="D12" s="7"/>
+      <c r="D12" s="7" t="s">
+        <v>20</v>
+      </c>
       <c r="E12" s="8"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -960,7 +962,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -977,7 +979,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -990,7 +992,7 @@
       </c>
       <c r="E15" s="8"/>
     </row>
-    <row r="16" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -1007,7 +1009,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -1015,10 +1017,12 @@
         <v>25</v>
       </c>
       <c r="C17" s="6"/>
-      <c r="D17" s="7"/>
+      <c r="D17" s="7" t="s">
+        <v>62</v>
+      </c>
       <c r="E17" s="8"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -1035,7 +1039,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="5">
         <v>17</v>
       </c>
@@ -1052,7 +1056,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="5">
         <v>18</v>
       </c>
@@ -1069,7 +1073,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="5">
         <v>19</v>
       </c>
@@ -1086,7 +1090,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="5">
         <v>20</v>
       </c>
@@ -1099,7 +1103,7 @@
       </c>
       <c r="E22" s="8"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="5">
         <v>21</v>
       </c>
@@ -1116,7 +1120,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="5">
         <v>22</v>
       </c>
@@ -1133,7 +1137,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="5">
         <v>23</v>
       </c>
@@ -1141,10 +1145,12 @@
         <v>10</v>
       </c>
       <c r="C25" s="6"/>
-      <c r="D25" s="7"/>
+      <c r="D25" s="7" t="s">
+        <v>17</v>
+      </c>
       <c r="E25" s="8"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="5">
         <v>24</v>
       </c>
@@ -1161,7 +1167,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="5">
         <v>25</v>
       </c>
@@ -1178,7 +1184,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="5">
         <v>26</v>
       </c>
@@ -1195,7 +1201,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="5">
         <v>27</v>
       </c>
@@ -1212,7 +1218,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="5">
         <v>28</v>
       </c>
@@ -1229,7 +1235,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="5">
         <v>29</v>
       </c>
@@ -1238,11 +1244,11 @@
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="7" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="E31" s="8"/>
     </row>
-    <row r="32" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" s="5">
         <v>30</v>
       </c>
@@ -1255,7 +1261,7 @@
       </c>
       <c r="E32" s="8"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="5">
         <v>31</v>
       </c>
@@ -1272,7 +1278,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="5">
         <v>32</v>
       </c>
@@ -1289,7 +1295,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="5">
         <v>33</v>
       </c>
@@ -1297,10 +1303,12 @@
         <v>45</v>
       </c>
       <c r="C35" s="6"/>
-      <c r="D35" s="7"/>
+      <c r="D35" s="7" t="s">
+        <v>17</v>
+      </c>
       <c r="E35" s="8"/>
     </row>
-    <row r="36" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="5">
         <v>34</v>
       </c>
@@ -1317,7 +1325,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="34" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A37" s="5">
         <v>35</v>
       </c>
@@ -1326,16 +1334,16 @@
       </c>
       <c r="C37" s="6"/>
       <c r="D37" s="7" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E37" s="8"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="5">
         <v>36</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>51</v>
@@ -1347,28 +1355,28 @@
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="5">
         <v>37</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C39" s="6"/>
       <c r="D39" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E39" s="8"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="5">
         <v>38</v>
       </c>
       <c r="B40" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="D40" s="7" t="s">
         <v>12</v>
@@ -1377,15 +1385,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="41" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="9">
         <v>39</v>
       </c>
       <c r="B41" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C41" s="10" t="s">
         <v>61</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>62</v>
       </c>
       <c r="D41" s="11" t="s">
         <v>52</v>
@@ -1395,7 +1403,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E41"/>
+  <autoFilter ref="A1:E41" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>